<commit_message>
Update pipeline: preserve raw NO_MOSQ_POOLED, add variable renames, include vision LLM alternative
- NO_MOSQ_POOLED is now passed through as-is from OCR (raw values preserved)
- Variable renames throughout for readability (ri/ci -> row_idx/col_idx, v -> raw, etc.)
- Add ollama_vision_pipeline.py: whole-page GPU approach via vision LLM
- Update output CSV/XLSX with latest run
</commit_message>
<xml_diff>
--- a/mosquito_surveillance_data.xlsx
+++ b/mosquito_surveillance_data.xlsx
@@ -579,7 +579,7 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>3-negles</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -687,7 +687,7 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>50-</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>50edge</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">

</xml_diff>